<commit_message>
Retires a share of existing capacity by vintage age
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/BUCLfCR/BUCLfCR Bool Use Cap Life for Retirments.xlsx
+++ b/InputData/ctrl-settings/BUCLfCR/BUCLfCR Bool Use Cap Life for Retirments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\BUCCLfCR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\BUCLfCR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74444D37-C7AC-42D7-A9F1-EB79F599540A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E449AE26-BFD8-4F00-B5BA-FF3ADC777D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{BE93E9B0-23D9-4599-AD62-4298B8CF7C84}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="8250" activeTab="1" xr2:uid="{BE93E9B0-23D9-4599-AD62-4298B8CF7C84}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>BUCLfCR Boolean Use Capacity Lifetime for Capacity Retirements</t>
   </si>
@@ -60,7 +60,79 @@
     <t>Retire plants at lifetime</t>
   </si>
   <si>
-    <t>1 = yes, 0 = no</t>
+    <t>hard coal</t>
+  </si>
+  <si>
+    <t>natural gas steam turbine</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle</t>
+  </si>
+  <si>
+    <t>nuclear</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>onshore wind</t>
+  </si>
+  <si>
+    <t>solar pv</t>
+  </si>
+  <si>
+    <t>solar thermal</t>
+  </si>
+  <si>
+    <t>biomass</t>
+  </si>
+  <si>
+    <t>geothermal</t>
+  </si>
+  <si>
+    <t>petroleum</t>
+  </si>
+  <si>
+    <t>natural gas peaker</t>
+  </si>
+  <si>
+    <t>lignite</t>
+  </si>
+  <si>
+    <t>offshore wind</t>
+  </si>
+  <si>
+    <t>crude oil</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
+  </si>
+  <si>
+    <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>hard coal w CCS</t>
+  </si>
+  <si>
+    <t>natural gas combined cycle w CCS</t>
+  </si>
+  <si>
+    <t>biomass w CCS</t>
+  </si>
+  <si>
+    <t>lignite w CCS</t>
+  </si>
+  <si>
+    <t>small modular reactor</t>
+  </si>
+  <si>
+    <t>hydrogen combustion turbine</t>
+  </si>
+  <si>
+    <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>boolean</t>
   </si>
 </sst>
 </file>
@@ -480,7 +552,7 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
@@ -490,12 +562,199 @@
       <c r="A1" t="s">
         <v>6</v>
       </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
         <v>0</v>
       </c>
     </row>

</xml_diff>